<commit_message>
extracted uS totals from ic raw data for sc exo comparison
</commit_message>
<xml_diff>
--- a/Data/GrabSample_data/RI23-uncertainty.xlsx
+++ b/Data/GrabSample_data/RI23-uncertainty.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="analytical-unceratinty" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="endmember-std" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="singletons" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -33,40 +34,40 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Analytical Uncertainty (Wanalytical​)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lab reports / instrument specs</t>
+    <t xml:space="preserve">Analytical uncertainty (W_analytical)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lab reports and instrument specs</t>
   </si>
   <si>
     <t xml:space="preserve">e.g., ±2% for ICP-OES, ±0.1‰ for δ18O.</t>
   </si>
   <si>
-    <t xml:space="preserve">End-member Std Dev (sem​)</t>
+    <t xml:space="preserve">End-member std dev (s_em)</t>
   </si>
   <si>
     <t xml:space="preserve">Your data</t>
   </si>
   <si>
-    <t xml:space="preserve">If you have multiple samples (e.g., 5 soil lysimeter samples), use their standard deviation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The "Single Sample" Case</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Genereux suggestion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If you only have one snow sample, you must use the Wanalytical​ or a "literature-derived" spatial variability estimate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PCA Loadings (Eigenvectors)</t>
+    <t xml:space="preserve">Standard deviation when we have multiple end-member samples for EMMA input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single measurement cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytical or literature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We use the W analytical or a literature-derived spatial variability estimate (Genereux 1998 suggestion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCA loadings (eigenvectors)</t>
   </si>
   <si>
     <t xml:space="preserve">pca.components_</t>
   </si>
   <si>
-    <t xml:space="preserve">Your existing code already generates this; you'll just need to extract it.</t>
+    <t xml:space="preserve">Produced as emma.py output</t>
   </si>
   <si>
     <t xml:space="preserve"># Analytical uncertainty for geochemical tracers in RI23 </t>
@@ -133,6 +134,30 @@
   </si>
   <si>
     <t xml:space="preserve">TOC mg_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Standard deviation for end-member selections for each event EMMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Event_ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseflow_EM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil_EM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melt_EM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wade_20230209</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wade_202303</t>
   </si>
 </sst>
 </file>
@@ -230,6 +255,10 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.12"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -391,6 +420,57 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>

</xml_diff>